<commit_message>
feat: Implement 6 core dashboard updates (Timeline revision segregation with SSR, country glance revision columns, 100% by-poll resolution, constituency-level booth voters, synchronized LGD-JOSHUA districts, 36 states/UTs)
</commit_message>
<xml_diff>
--- a/static/data/exports/Retro_AS_AE_2011.xlsx
+++ b/static/data/exports/Retro_AS_AE_2011.xlsx
@@ -1470,11 +1470,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E17" t="n">
         <v>6234</v>
@@ -6855,11 +6855,11 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>1724504</v>
+        <v>1724505</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Jamal Uddin Choudhury</t>
+          <t>Motiur Rahman Barbhuiya</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6892,7 +6892,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Jamal Uddin Choudhury</t>
+          <t>Motiur Rahman Barbhuiya</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -6917,11 +6917,11 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>1724505</v>
+        <v>1724504</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Motiur Rahman Barbhuiya</t>
+          <t>Jamal Uddin Choudhury</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -6954,7 +6954,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Motiur Rahman Barbhuiya</t>
+          <t>Jamal Uddin Choudhury</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7448,11 +7448,11 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E113" t="n">
         <v>6163</v>
@@ -18725,11 +18725,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E293" t="n">
         <v>22151</v>
@@ -19221,11 +19221,11 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E301" t="n">
         <v>2844</v>
@@ -22259,11 +22259,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E350" t="n">
         <v>20609</v>
@@ -24615,11 +24615,11 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E388" t="n">
         <v>6450</v>
@@ -25226,20 +25226,20 @@
     </row>
     <row r="398">
       <c r="A398" t="n">
-        <v>1724799</v>
+        <v>1724798</v>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Azmul Hoque</t>
+          <t>Md Jalal Uddin Ali</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>AIMF</t>
+          <t>AGP</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>19896</v>
+        <v>19864</v>
       </c>
       <c r="E398" t="n">
         <v>772</v>
@@ -25263,12 +25263,12 @@
       </c>
       <c r="K398" t="inlineStr">
         <is>
-          <t>Azmul Hoque</t>
+          <t>Md Jalal Uddin Ali</t>
         </is>
       </c>
       <c r="L398" t="inlineStr">
         <is>
-          <t>AIMF</t>
+          <t>AGP</t>
         </is>
       </c>
       <c r="Q398" t="b">
@@ -25288,20 +25288,20 @@
     </row>
     <row r="399">
       <c r="A399" t="n">
-        <v>1724798</v>
+        <v>1724799</v>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Md Jalal Uddin Ali</t>
+          <t>Azmul Hoque</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>AGP</t>
+          <t>AIMF</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>19864</v>
+        <v>19896</v>
       </c>
       <c r="E399" t="n">
         <v>772</v>
@@ -25325,12 +25325,12 @@
       </c>
       <c r="K399" t="inlineStr">
         <is>
-          <t>Md Jalal Uddin Ali</t>
+          <t>Azmul Hoque</t>
         </is>
       </c>
       <c r="L399" t="inlineStr">
         <is>
-          <t>AGP</t>
+          <t>AIMF</t>
         </is>
       </c>
       <c r="Q399" t="b">
@@ -25731,11 +25731,11 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D406" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E406" t="n">
         <v>8517</v>
@@ -28521,11 +28521,11 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D451" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E451" t="n">
         <v>3314</v>
@@ -31807,11 +31807,11 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D504" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E504" t="n">
         <v>23274</v>
@@ -32985,11 +32985,11 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D523" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E523" t="n">
         <v>4613</v>
@@ -37945,11 +37945,11 @@
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D603" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E603" t="n">
         <v>1903</v>
@@ -39061,11 +39061,11 @@
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D621" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E621" t="n">
         <v>7795</v>
@@ -39557,11 +39557,11 @@
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D629" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E629" t="n">
         <v>32362</v>
@@ -46654,11 +46654,11 @@
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D742" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E742" t="n">
         <v>1577</v>
@@ -55458,11 +55458,11 @@
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D884" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E884" t="n">
         <v>2033</v>
@@ -58868,11 +58868,11 @@
       </c>
       <c r="C939" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D939" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E939" t="n">
         <v>2699</v>
@@ -61286,11 +61286,11 @@
       </c>
       <c r="C978" t="inlineStr">
         <is>
-          <t>CPM</t>
+          <t>CPI(M)</t>
         </is>
       </c>
       <c r="D978" t="n">
-        <v>19912</v>
+        <v>19875</v>
       </c>
       <c r="E978" t="n">
         <v>4116</v>

</xml_diff>